<commit_message>
Served first set of interrogatories update content of 3 RFAs
</commit_message>
<xml_diff>
--- a/OffenseStrategies/Estimates/DamagedWindowsFromPrievePhotos.xlsx
+++ b/OffenseStrategies/Estimates/DamagedWindowsFromPrievePhotos.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/billlu/Projects/FarmersInsurance-github/OffenseStrategies/Estimates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71AF8C5D-A414-0049-9A78-05A8A28EE5A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{963A0D27-86AD-9640-BAC8-5598E1131F4C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="56920" yWindow="3420" windowWidth="27140" windowHeight="18400" xr2:uid="{6BADC156-4335-9445-B56E-769EE49F1A3A}"/>
+    <workbookView xWindow="45820" yWindow="3200" windowWidth="27140" windowHeight="18400" xr2:uid="{6BADC156-4335-9445-B56E-769EE49F1A3A}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -424,7 +424,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -434,12 +434,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="0" tint="-4.9989318521683403E-2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.59999389629810485"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -481,15 +475,17 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -512,14 +508,14 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>2</xdr:col>
+      <xdr:col>1</xdr:col>
       <xdr:colOff>76200</xdr:colOff>
       <xdr:row>9</xdr:row>
       <xdr:rowOff>101600</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>1231900</xdr:colOff>
+      <xdr:colOff>317500</xdr:colOff>
       <xdr:row>9</xdr:row>
       <xdr:rowOff>627391</xdr:rowOff>
     </xdr:to>
@@ -874,706 +870,685 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BB71EE3E-1567-0942-83C2-0818924E2DD9}">
-  <dimension ref="A1:F48"/>
+  <dimension ref="A1:E48"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="41.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="21.33203125" customWidth="1"/>
-    <col min="4" max="4" width="22.33203125" customWidth="1"/>
-    <col min="5" max="5" width="30.5" customWidth="1"/>
-    <col min="6" max="6" width="55.33203125" customWidth="1"/>
+    <col min="1" max="1" width="35" customWidth="1"/>
+    <col min="2" max="2" width="12" customWidth="1"/>
+    <col min="3" max="3" width="16.1640625" customWidth="1"/>
+    <col min="4" max="4" width="20" customWidth="1"/>
+    <col min="5" max="5" width="31.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1" s="4" t="s">
+        <v>0</v>
+      </c>
       <c r="B1" s="4" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="F1" s="4" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A2" s="5"/>
+    <row r="2" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>4</v>
+      </c>
       <c r="B2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C2" t="s">
         <v>5</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="C2" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="E2" s="9">
+      <c r="D2" s="8">
         <v>7602.17</v>
       </c>
-      <c r="F2" t="s">
+      <c r="E2" s="9" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A3" s="5"/>
+    <row r="3" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>9</v>
+      </c>
       <c r="B3" t="s">
-        <v>9</v>
-      </c>
-      <c r="C3" t="s">
         <v>10</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="C3" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="E3" s="9">
+      <c r="D3" s="8">
         <v>7602.17</v>
       </c>
-      <c r="F3" t="s">
+      <c r="E3" s="9" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A4" s="5"/>
-      <c r="B4" t="s">
+    <row r="4" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
         <v>12</v>
       </c>
-      <c r="D4" s="3"/>
-      <c r="E4" s="9">
+      <c r="C4" s="3"/>
+      <c r="D4" s="8">
         <v>7085.76</v>
       </c>
-      <c r="F4" t="s">
+      <c r="E4" s="9" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A5" s="5"/>
-      <c r="B5" t="s">
+    <row r="5" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
         <v>14</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="C5" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="E5" s="9">
+      <c r="D5" s="8">
         <v>13311.3</v>
       </c>
-      <c r="F5" t="s">
+      <c r="E5" s="9" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A6" s="5"/>
-      <c r="B6" t="s">
+    <row r="6" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
         <v>17</v>
       </c>
-      <c r="D6" s="3" t="s">
+      <c r="C6" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="E6" s="9">
+      <c r="D6" s="8">
         <v>7602.17</v>
       </c>
-      <c r="F6" t="s">
+      <c r="E6" s="9" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="D7" s="3"/>
-      <c r="E7" s="2"/>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="D8" s="3"/>
-      <c r="E8" s="2"/>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A9" s="5"/>
-      <c r="B9" t="s">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="C7" s="3"/>
+      <c r="D7" s="2"/>
+      <c r="E7" s="9"/>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="C8" s="3"/>
+      <c r="D8" s="2"/>
+      <c r="E8" s="9"/>
+    </row>
+    <row r="9" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
         <v>20</v>
       </c>
-      <c r="D9" s="3" t="s">
+      <c r="C9" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="E9" s="9">
+      <c r="D9" s="8">
         <v>8025.57</v>
       </c>
-      <c r="F9" t="s">
+      <c r="E9" s="9" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="10" spans="1:6" ht="56" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="5"/>
-      <c r="B10" t="s">
+    <row r="10" spans="1:5" ht="56" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
         <v>21</v>
       </c>
-      <c r="D10" s="3"/>
-      <c r="E10" s="9">
+      <c r="C10" s="3"/>
+      <c r="D10" s="8">
         <v>6686.91</v>
       </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A11" s="5"/>
-      <c r="B11" t="s">
+      <c r="E10" s="9"/>
+    </row>
+    <row r="11" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
         <v>24</v>
       </c>
-      <c r="D11" s="3" t="s">
+      <c r="C11" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="E11" s="9">
+      <c r="D11" s="8">
         <v>7602.21</v>
       </c>
-      <c r="F11" t="s">
+      <c r="E11" s="9" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="D12" s="3"/>
-      <c r="E12" s="2"/>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A13" s="5"/>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="C12" s="3"/>
+      <c r="D12" s="2"/>
+      <c r="E12" s="9"/>
+    </row>
+    <row r="13" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>25</v>
+      </c>
       <c r="B13" t="s">
-        <v>25</v>
-      </c>
-      <c r="C13" t="s">
         <v>28</v>
       </c>
-      <c r="D13" s="3" t="s">
+      <c r="C13" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="E13" s="9">
+      <c r="D13" s="8">
         <v>2493.48</v>
       </c>
-      <c r="F13" t="s">
+      <c r="E13" s="9" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A14" s="5"/>
+    <row r="14" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>108</v>
+      </c>
       <c r="B14" t="s">
-        <v>108</v>
-      </c>
-      <c r="C14" t="s">
         <v>109</v>
       </c>
-      <c r="D14" s="3" t="s">
+      <c r="C14" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="E14" s="9">
+      <c r="D14" s="8">
         <v>2493.48</v>
       </c>
-      <c r="F14" t="s">
+      <c r="E14" s="9" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A15" s="5"/>
+    <row r="15" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>29</v>
+      </c>
       <c r="B15" t="s">
-        <v>29</v>
-      </c>
-      <c r="C15" t="s">
         <v>30</v>
       </c>
-      <c r="D15" s="3" t="s">
+      <c r="C15" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="E15" s="9">
+      <c r="D15" s="8">
         <v>7957.75</v>
       </c>
-      <c r="F15" t="s">
+      <c r="E15" s="9" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A16" s="5"/>
+    <row r="16" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>33</v>
+      </c>
       <c r="B16" t="s">
-        <v>33</v>
-      </c>
-      <c r="C16" t="s">
         <v>34</v>
       </c>
-      <c r="D16" s="3" t="s">
+      <c r="C16" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="E16" s="9">
+      <c r="D16" s="8">
         <v>7957.75</v>
       </c>
-      <c r="F16" t="s">
+      <c r="E16" s="9" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A17" s="5"/>
+    <row r="17" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>37</v>
+      </c>
       <c r="B17" t="s">
-        <v>37</v>
-      </c>
-      <c r="C17" t="s">
         <v>40</v>
       </c>
-      <c r="D17" s="3" t="s">
+      <c r="C17" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="E17" s="9">
+      <c r="D17" s="8">
         <v>2493.48</v>
       </c>
-      <c r="F17" t="s">
+      <c r="E17" s="9" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A18" s="5"/>
+    <row r="18" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>39</v>
+      </c>
       <c r="B18" t="s">
-        <v>39</v>
-      </c>
-      <c r="C18" t="s">
         <v>41</v>
       </c>
-      <c r="D18" s="3" t="s">
+      <c r="C18" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="E18" s="9">
+      <c r="D18" s="8">
         <v>2493.48</v>
       </c>
-      <c r="F18" t="s">
+      <c r="E18" s="9" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A19" s="5"/>
+    <row r="19" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
+        <v>50</v>
+      </c>
       <c r="B19" t="s">
-        <v>50</v>
-      </c>
-      <c r="C19" t="s">
         <v>51</v>
       </c>
-      <c r="D19" s="3" t="s">
+      <c r="C19" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="E19" s="9">
+      <c r="D19" s="8">
         <v>1693.95</v>
       </c>
-      <c r="F19" t="s">
+      <c r="E19" s="9" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A20" s="5"/>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
+        <v>54</v>
+      </c>
       <c r="B20" t="s">
-        <v>54</v>
-      </c>
-      <c r="C20" t="s">
         <v>55</v>
       </c>
-      <c r="D20" s="3" t="s">
+      <c r="C20" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="E20" s="9">
+      <c r="D20" s="8">
         <f>1693.95*4</f>
         <v>6775.8</v>
       </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A21" s="5"/>
+      <c r="E20" s="9"/>
+    </row>
+    <row r="21" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
+        <v>47</v>
+      </c>
       <c r="B21" t="s">
-        <v>47</v>
-      </c>
-      <c r="C21" t="s">
         <v>111</v>
       </c>
-      <c r="D21" s="3" t="s">
+      <c r="C21" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="E21" s="9">
+      <c r="D21" s="8">
         <v>2525.98</v>
       </c>
-      <c r="F21" t="s">
+      <c r="E21" s="9" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A22" s="5"/>
+    <row r="22" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
+        <v>112</v>
+      </c>
       <c r="B22" t="s">
-        <v>112</v>
-      </c>
-      <c r="C22" t="s">
         <v>113</v>
       </c>
-      <c r="D22" s="3" t="s">
+      <c r="C22" s="3" t="s">
         <v>116</v>
       </c>
-      <c r="E22" s="9">
+      <c r="D22" s="8">
         <v>9927.32</v>
       </c>
-      <c r="F22" t="s">
+      <c r="E22" s="9" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A23" s="5"/>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A23" t="s">
+        <v>115</v>
+      </c>
       <c r="B23" t="s">
-        <v>115</v>
-      </c>
-      <c r="C23" t="s">
         <v>114</v>
       </c>
-      <c r="D23" s="3" t="s">
+      <c r="C23" s="3" t="s">
         <v>116</v>
       </c>
-      <c r="E23" s="9">
+      <c r="D23" s="8">
         <v>9927.32</v>
       </c>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A24" s="5"/>
+      <c r="E23" s="9"/>
+    </row>
+    <row r="24" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="A24" t="s">
+        <v>56</v>
+      </c>
       <c r="B24" t="s">
-        <v>56</v>
-      </c>
-      <c r="C24" t="s">
         <v>58</v>
       </c>
-      <c r="D24" s="3" t="s">
+      <c r="C24" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="E24" s="9">
+      <c r="D24" s="8">
         <v>2525.98</v>
       </c>
-      <c r="F24" t="s">
+      <c r="E24" s="9" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A25" s="5"/>
+    <row r="25" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="A25" t="s">
+        <v>59</v>
+      </c>
       <c r="B25" t="s">
-        <v>59</v>
-      </c>
-      <c r="C25" t="s">
         <v>63</v>
       </c>
-      <c r="D25" s="3" t="s">
+      <c r="C25" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="E25" s="9">
+      <c r="D25" s="8">
         <v>3205.31</v>
       </c>
-      <c r="F25" t="s">
+      <c r="E25" s="9" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A26" s="5"/>
+    <row r="26" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="A26" t="s">
+        <v>62</v>
+      </c>
       <c r="B26" t="s">
-        <v>62</v>
-      </c>
-      <c r="C26" t="s">
         <v>64</v>
       </c>
-      <c r="D26" s="3" t="s">
+      <c r="C26" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="E26" s="9">
+      <c r="D26" s="8">
         <v>2525.98</v>
       </c>
-      <c r="F26" t="s">
+      <c r="E26" s="9" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A27" s="5"/>
+    <row r="27" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="A27" t="s">
+        <v>92</v>
+      </c>
       <c r="B27" t="s">
-        <v>92</v>
-      </c>
-      <c r="C27" t="s">
         <v>67</v>
       </c>
-      <c r="D27" s="3" t="s">
+      <c r="C27" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="E27" s="9">
+      <c r="D27" s="8">
         <v>2576.7199999999998</v>
       </c>
-      <c r="F27" t="s">
+      <c r="E27" s="9" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A28" s="5"/>
+    <row r="28" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="A28" t="s">
+        <v>91</v>
+      </c>
       <c r="B28" t="s">
-        <v>91</v>
-      </c>
-      <c r="C28" t="s">
         <v>93</v>
       </c>
-      <c r="D28" s="3" t="s">
+      <c r="C28" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="E28" s="9">
+      <c r="D28" s="8">
         <v>2355.16</v>
       </c>
-      <c r="F28" t="s">
+      <c r="E28" s="9" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A29" s="5"/>
+    <row r="29" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+      <c r="A29" t="s">
+        <v>69</v>
+      </c>
       <c r="B29" t="s">
-        <v>69</v>
-      </c>
-      <c r="C29" t="s">
         <v>71</v>
       </c>
-      <c r="D29" s="3" t="s">
+      <c r="C29" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="E29" s="9">
+      <c r="D29" s="8">
         <v>2525.98</v>
       </c>
-      <c r="F29" t="s">
+      <c r="E29" s="9" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A30" s="5"/>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A30" t="s">
+        <v>72</v>
+      </c>
       <c r="B30" t="s">
-        <v>72</v>
-      </c>
-      <c r="C30" t="s">
         <v>73</v>
       </c>
-      <c r="D30" s="3" t="s">
+      <c r="C30" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="E30" s="9">
+      <c r="D30" s="8">
         <v>3135.92</v>
       </c>
-    </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A31" s="5"/>
+      <c r="E30" s="9"/>
+    </row>
+    <row r="31" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="A31" t="s">
+        <v>75</v>
+      </c>
       <c r="B31" t="s">
-        <v>75</v>
-      </c>
-      <c r="C31" t="s">
         <v>76</v>
       </c>
-      <c r="D31" s="3" t="s">
+      <c r="C31" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="E31" s="9">
+      <c r="D31" s="8">
         <v>2525.98</v>
       </c>
-      <c r="F31" t="s">
+      <c r="E31" s="9" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A32" s="5"/>
+    <row r="32" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="A32" t="s">
+        <v>78</v>
+      </c>
       <c r="B32" t="s">
+        <v>79</v>
+      </c>
+      <c r="C32" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="D32" s="8">
+        <v>5434.84</v>
+      </c>
+      <c r="E32" s="9" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A33" t="s">
         <v>78</v>
       </c>
-      <c r="C32" t="s">
-        <v>79</v>
-      </c>
-      <c r="D32" s="3" t="s">
+      <c r="B33" t="s">
+        <v>81</v>
+      </c>
+      <c r="C33" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="E32" s="9">
+      <c r="D33" s="8">
         <v>5434.84</v>
       </c>
-      <c r="F32" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A33" s="5"/>
-      <c r="B33" t="s">
-        <v>78</v>
-      </c>
-      <c r="C33" t="s">
-        <v>81</v>
-      </c>
-      <c r="D33" s="3" t="s">
-        <v>80</v>
-      </c>
-      <c r="E33" s="9">
-        <v>5434.84</v>
-      </c>
-      <c r="F33" t="s">
+      <c r="E33" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A34" s="6"/>
-      <c r="B34" s="6" t="s">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A34" s="5" t="s">
         <v>84</v>
       </c>
-      <c r="C34" s="6" t="s">
+      <c r="B34" s="5" t="s">
         <v>90</v>
       </c>
-      <c r="D34" s="7"/>
-      <c r="E34" s="8" t="s">
+      <c r="C34" s="6"/>
+      <c r="D34" s="7" t="s">
         <v>85</v>
       </c>
-      <c r="F34" s="6" t="s">
+      <c r="E34" s="5" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A35" s="6"/>
-      <c r="B35" s="6" t="s">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A35" s="5" t="s">
         <v>88</v>
       </c>
-      <c r="C35" s="6" t="s">
+      <c r="B35" s="5" t="s">
         <v>89</v>
       </c>
-      <c r="D35" s="7"/>
-      <c r="E35" s="8" t="s">
+      <c r="C35" s="6"/>
+      <c r="D35" s="7" t="s">
         <v>85</v>
       </c>
-      <c r="F35" s="6" t="s">
+      <c r="E35" s="5" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A36" s="5"/>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A36" t="s">
+        <v>95</v>
+      </c>
       <c r="B36" t="s">
-        <v>95</v>
-      </c>
-      <c r="C36" t="s">
         <v>96</v>
       </c>
-      <c r="D36" s="3" t="s">
+      <c r="C36" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="E36" s="9">
+      <c r="D36" s="8">
         <v>7602.17</v>
       </c>
-      <c r="F36" t="s">
+      <c r="E36" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A37" s="5"/>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A37" t="s">
+        <v>98</v>
+      </c>
       <c r="B37" t="s">
-        <v>98</v>
-      </c>
-      <c r="C37" t="s">
         <v>99</v>
       </c>
-      <c r="D37" s="3" t="s">
+      <c r="C37" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="E37" s="9">
+      <c r="D37" s="8">
         <v>7602.17</v>
       </c>
-      <c r="F37" t="s">
+      <c r="E37" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A38" s="5"/>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A38" t="s">
+        <v>101</v>
+      </c>
       <c r="B38" t="s">
-        <v>101</v>
-      </c>
-      <c r="C38" t="s">
         <v>103</v>
       </c>
-      <c r="D38" s="3" t="s">
+      <c r="C38" s="3" t="s">
         <v>104</v>
       </c>
-      <c r="E38" s="9">
+      <c r="D38" s="8">
         <v>4762.38</v>
       </c>
-      <c r="F38" t="s">
+      <c r="E38" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A39" s="5"/>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A39" t="s">
+        <v>105</v>
+      </c>
       <c r="B39" t="s">
-        <v>105</v>
-      </c>
-      <c r="C39" t="s">
         <v>106</v>
       </c>
-      <c r="D39" s="3" t="s">
+      <c r="C39" s="3" t="s">
         <v>104</v>
       </c>
-      <c r="E39" s="9">
+      <c r="D39" s="8">
         <v>4762.38</v>
       </c>
-      <c r="F39" t="s">
+      <c r="E39" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="D40" s="3"/>
-      <c r="E40" s="2"/>
-    </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="B41" t="s">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="C40" s="3"/>
+      <c r="D40" s="2"/>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A41" t="s">
         <v>118</v>
       </c>
-      <c r="D41" s="3"/>
-      <c r="E41" s="2">
+      <c r="C41" s="3"/>
+      <c r="D41" s="2">
         <v>7602.17</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="B42" t="s">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A42" t="s">
         <v>119</v>
       </c>
-      <c r="D42" s="3"/>
-      <c r="E42" s="2">
+      <c r="C42" s="3"/>
+      <c r="D42" s="2">
         <f>2240.49*2</f>
         <v>4480.9799999999996</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="D43" s="3"/>
-      <c r="E43" s="2"/>
-    </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="B44" t="s">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="C43" s="3"/>
+      <c r="D43" s="2"/>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A44" t="s">
         <v>42</v>
       </c>
-      <c r="D44" s="3"/>
-      <c r="E44" s="2">
+      <c r="C44" s="3"/>
+      <c r="D44" s="2">
         <v>51253.02</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="B45" t="s">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A45" t="s">
         <v>43</v>
       </c>
-      <c r="E45" s="2">
+      <c r="D45" s="2">
         <v>10500.93</v>
       </c>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="B46" t="s">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A46" t="s">
         <v>44</v>
       </c>
-      <c r="E46" s="2">
+      <c r="D46" s="2">
         <v>3404.7</v>
       </c>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="B47" t="s">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A47" t="s">
         <v>117</v>
       </c>
-      <c r="E47" s="2">
+      <c r="D47" s="2">
         <v>2054.6999999999998</v>
       </c>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="E48" s="1">
-        <f>SUM(E2:E47)</f>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="D48" s="1">
+        <f>SUM(D2:D47)</f>
         <v>258530.36000000007</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="landscape" horizontalDpi="0" verticalDpi="0"/>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
+<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
+  <clbl:label id="{1712afef-9f4e-4511-a60c-36df6704e051}" enabled="1" method="Standard" siteId="{4e9dbbfb-394a-4583-8810-53f81f819e3b}" contentBits="0" removed="0"/>
+</clbl:labelList>
 </file>
</xml_diff>